<commit_message>
feat(server): yfinance data cache
</commit_message>
<xml_diff>
--- a/server/src/datasource/data_j_service_ai_consulting_candidates.xlsx
+++ b/server/src/datasource/data_j_service_ai_consulting_candidates.xlsx
@@ -413,9 +413,677 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>company_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>yahoo_ticker</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>industry</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>matched_ai_keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ＮＪＳ</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2325.T</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.njs.co.jp</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Waste Management</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NJS Co., Ltd., together with its subsidiaries, primarily engages in water and environmental consulting, digital transformation, and customer services business in Japan and internationally. It provides community and environmental solutions, including global environmental, water environment, urban development, and disaster prevention and mitigation solutions; infrastructure solutions comprising survey and planning of water supply and sewerage system, pipeline, treatment plant, infrastructure management, and management consulting; and survey and planning, infrastructure development, and operational capacity building support services. The company also offers software, system construction and operation services, infrastructure management services, disaster prevention and mitigation, business operations, and AI utilization system; develops drones, robotics, sensors, and data analysis used for inspection; and customer service, such as information dissemination, customer relations, and communication services. The company was formerly known as Nippon Jogesuido Sekkei Co., Ltd. and changed its name to NJS Co., Ltd. in April 2015. NJS Co., Ltd. was incorporated in 1951 and is headquartered in Tokyo, Japan.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>グローカルマーケティング</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>266A.T</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://glocal-marketing.jp</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Specialty Business Services</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Glocal Marketing Co., Ltd. engages in marketing support, and human resource recruitment and development support businesses in Japan. The company offers marketing and sales consulting, seminars and training, marketing research, SNS utilization support, Google ads, SNS advertising operation support, and press release creation support services; photography, video production, flyer, pamphlet, etc. design production; customer management system and implementation support services. It also provides strategy design support seminars and
+training support for formulating personnel evaluation systems; and drafting and creating a DX promotion roadmap AI, implementation consulting, and groupware implementation consulting service, as well as planning and implementation of events for child-rearing families. The company was incorporated in 2020 and is headquartered in Nagaoka, Japan.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>サイバーエージェント</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4751.T</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.cyberagent.co.jp</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Advertising Agencies</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CyberAgent, Inc., together with its subsidiaries, engages in the internet advertising business in Japan. It operates through Media Business, Internet Advertising Business, Game Business, Investment Development Business, and Other Businesses segments. The company operates Ameba, a video streaming platform with various channels, including 24-hour news, dramas, romance shows, anime, and sports; and WinTicket for internet betting for sports events, such as horse, bicycle, and auto racing, as well as fan community app development and service management; IP works and content; performance; merchandising; and overseas marketing. It also offers AI solutions; creative production; DX business; research and consulting; and smartphone games. In addition, the company engages in news content planning and production; smartphone advertising; creative office planning and management; corporate venture capital; fund establishment and management; crowdfunding; and management of professional soccer teams. CyberAgent, Inc. was incorporated in 1998 and is headquartered in Shibuya, Japan.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ＳＯＬＩＺＥ　Ｈｏｌｄｉｎｇｓ</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5871.T</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.solize.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Computer Hardware</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SOLIZE Corporation, together with its subsidiaries, provides digital engineering services in Japan, North America, China, India, Thailand, Europe, and internationally. It operates in two segments, Design Business and Manufacturing Business. The company engages in digital engineering development support services, including 3D digital tools, styling, design, analysis, XR, and AI; 3D printer parts manufacturing, such as online 3D printing, 3D printer prototype and final product production, and research and development support; 3D printer sales and maintenance; and transformation consulting services for car, energy infrastructure, construction/general contractor, and LCA. It also provides AI comprising SpectA KY-tool, RFQ guide view, and DKM, as well as mathematics and data scientist-type generative AI agent development services; SDV, which includes MBD/MBSE, autonomous driving, and thermal management; cybersecurity and digital forensics; software development services for embedded control and business systems; educational services, such as private after-school care management, after-school care management consulting, after-school care staff training, and human resource development; and business solutions/DX support. The company was incorporated in 1990 and is headquartered in Chiyoda, Japan.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ai, generative ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>イー・ガーディアン</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>6050.T</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.e-guardian.co.jp</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>E-Guardian Inc. provides Internet security services in Japan, Singapore, and internationally. The company offers consulting, AI solutions, cyber security, debugging, rating, web content monitoring, advertisement review and operation support, customer support, social media, and global services. E-Guardian Inc. was incorporated in 1998 and is headquartered in Minato, Japan.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>メタリアル</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6182.T</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.metareal.jp</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>MetaReal Corporation develops, administers, and sells AI automatic translation services. It offers industry-specific AI development and implementation consulting services; language-free service with automatic translation; and VR Services, as well as wearable devices for construction industry; and VR-related products and solutions. It also provides Metareal AI, a document management AI; Work Done AI Series; Public Relations AI; Quarterly report API; Rakuyaku AI, a pharmaceuticals large-scale language model; and ella, character AI translation engine. In addition, the company offers AI automatic translation, such as T-4OO, and Onyaku; and metaverse services, including STUDIO55, and Digital Twin. The company was formerly known as Rozetta Corp. and changed its name to MetaReal Corporation in September 2021. MetaReal Corporation was incorporated in 1952 and is headquartered in Tokyo, Japan.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>バーチャレクス・ホールディングス</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>6193.T</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.vx-holdings.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Virtualex Holdings, Inc., through its subsidiaries, engages in IT and consulting, and outsourcing business in Japan and internationally. The company is involved in contact center operation; acts as generalists; onsite team engineering, offshore development, and IT operation outsourcing businesses; research and development, and acquisition of new technology and solution. It also provides consultation, outsourcing, and CRM software development services; web system, educational solution, and research and development related to AI; operational base for contact center outsourcing and BPO service; and digital marketing services. The company was formerly known as Virtualex Consulting, Inc. and changed its name to Virtualex Holdings, Inc. in October 2017. Virtualex Holdings, Inc. was incorporated in 1999 and is headquartered in Minato, Japan.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>6200.T</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.insource.co.jp</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Education &amp; Training Services</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Insource Co., Ltd. provides various lecturer dispatch type training, open lecture, and other services in Japan. It offers on-site training; open seminars; educational; IT services; and engages other businesses, such as e-learning/video production, online seminar administration services, video training content, workshop and consulting services, DX promotion support, AI/ RPA introduction support, online seminar agency, and recruitment services. Insource Co., Ltd. was founded in 2002 and is headquartered in Tokyo, Japan.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ベイカレント</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>6532.T</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.baycurrent.co.jp</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Consulting Services</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Baycurrent, Inc. provides consulting services in Japan. It offers AI, transformation, sustainability GX, strategy and corporate finance, customer experience, digital technology, data analytics, technology innovation, global business, marketing and sales, M&amp;A, supply chain and operations, intelligent automation, talent and organization, cost management, engineering and manufacturing, cloud, digital commerce, infrastructure, security, and managed services. The company also engages in the IT consulting and implementation; system consulting and integration; and management and operations activities. It serves high tech, media and entertainment, telecommunications, mobility, healthcare, retail, consumer products and distribution, industrial machinery, bank and payments, capital markets, insurance, energy, materials, chemicals and plants, transportation and logistics, developer, general trading company, and aerospace and defense industries. Baycurrent, Inc. was formerly known as BayCurrent Consulting, Inc and changed its name as BayCurrent, Inc. in September 2024. The company was founded in 1998 and is based in Tokyo, Japan.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>エスユーエス</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>6554.T</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.sus-g.co.jp</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Conglomerates</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SUS Co.,Ltd. engages in the worker dispatching business in Japan. The company provides engineer dispatch and development contracts in the fields of IT, mechanical, electrical, chemical, and biological; AI education and solutions; AR/VR education, solution development, and sales; IT consulting, system development, and implementation support in the ERP field; HR consulting and technology; and other IT-based services. It also offers various products, such as XR Solution; SUS Lab; VR Innovation Academy Kyoto; AI designer training course; and SUZAKU, a talent management system. The company was formerly known as Japan Staff Leasing Co., Ltd. and changed its name to SUS Co.,Ltd. in October 2013. SUS Co.,Ltd. was incorporated in 1999 and is headquartered in Kyoto, Japan.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ＴＤＳＥ</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>7046.T</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.tdse.jp</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>TDSE Inc. primarily provides consulting services on information processing and computer systems in Japan. The company offers DX and analytics consulting, SNS analysis, analysis base construction, and analysis operation and application development services; and IoT data utilization, learning utilization, and data scientist development support services. It also provides Scorobo, an artificial intelligence engine for use in finance, digital marketing, manufacture, social infrastructure, human resources, and telematics industries; and NetBase, a social listening tool for enterprise social analytics. The company was formerly known as Tecnos Data Science Engineering Incorporated and changed its name to TDSE Inc. in November 2021. TDSE Inc. was incorporated in 2013 and is based in Tokyo, Japan.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>artificial intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ピアズ</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>7066.T</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.peers.jp</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Conglomerates</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Peers Co.,Ltd. provides consulting solutions. provides consulting services offers three main services: sales promotion, online customer service, and AI boarding. The company supports digital transformation to achieve labor-saving and automation in store operations, provides online customer service systems to stores, and offers comprehensive human resource development support services in the sales field. It offers Onlinx, an online customer service system; video call center systems; Mimik, a training AI system to analyze facial expressions and emotions; online customer service center management; and RemoteworkBOX, a service to reserve a private booth in the city with a smartphone. The company also provides education training; consulting services; sales promotion services, such as in-store events and operational improvements at sales sites; and professional personnel staffing services. Peers Co.,Ltd. was incorporated in 2002 and is headquartered in Tokyo, Japan.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>デリバリーコンサルティング</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>9240.T</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.deliv.co.jp</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Delivery Consulting Inc. provides technology solutions consulting services in Japan and internationally. The company offers data infrastructure architecture and cloud migration, IoT data architecture, and data security governance; system modernization; dashboard design, data modeling and engineering, and data application, as well as support for in-house production; intelligent automation; solution engineering; system architecture and application development; cloud strategy and migration; data strategy; AI and analytics; modernization diagnostics and in-house consulting services; and data managed services. It also provides contact center reform and AI at customer contact points to optimize the customer experience through digital utilization. In addition, the company offers Salesforce Sales Cloud; Wordsmith, a natural language generation engine; and Tableau, a BI tool. Delivery Consulting Inc. was incorporated in 2003 and is headquartered in Tokyo, Japan.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>デジタリフト</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>9244.T</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://digitalift.co.jp</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Advertising Agencies</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>DIGITALIFT Inc. engages in the integrated digital marketing business in Japan. The company focuses on advertising and consulting services, as well as brand and media services. It provides marketing growth design solutions, includes digital advertising operations, affiliate management, SNS account creation and operation service, influencer marketing, and SEO/LLMO and business efficiency support; content equity enhancement solutions, such as website production and operation, owned media construction and recruitment support; data growth acceleration comprises dashboard building support, data-driven marketing development support, CRM strategy planning and execution, and AI-based marketing support solutions. The company was formerly known as Dencco, inc. and changed its name to DIGITALIFT Inc. in March 2020. DIGITALIFT Inc. was incorporated in 2012 and is based in Shibuya, Japan.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>プロジェクトホールディングス</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>9246.T</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://phd.co.jp</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Consulting Services</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ProjectHoldings, Inc. engages in the provision of digital transformation services in Japan. The company provides consulting services to develop new business and existing business transformation through digital transformation. It also offers AI consulting services for organizational support, strategy formulation support, and generative AI support. In addition, the company provides UIscope services, a usability testing service that improves UI/UX by recording the operations of test users; support for SNS operations, such as X and Instagram, website improvement, and marketing; SNS management support; and digital marketing services. Further, it offers technology services that support system development, operation and maintenance work, and software testing work; and healthcare services to corporate human resources departments. The company was formerly known as ProjectCompany, Inc. and changed its name to ProjectHoldings, Inc. in December 2023. The company was incorporated in 2016 and is headquartered in Minato, Japan.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ai, generative ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ＧＲＣＳ</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>9250.T</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.grcs.co.jp</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Information Technology Services</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>GRCS Inc. provides governance, risk, and compliance (GRC), and security solutions in Japan. The company offers Enterprise Risk MT, an ERM tool that provides company-wide risk management; Supplier Risk MT, a cloud application that streamlines outsourcing management and business partner management; OneTrust, a data privacy solution; Simple R, which links the learning management and ID management systems; and Connected Risk GRC Solution Audit Module, an audit management cloud solution. It also provides CSIRT MT.mss, a cloud application that enables CSIRTs within companies and organizations to respond to incidents and vulnerabilities; Vulnerability TODAY, an email distribution service that collect vulnerability information; Netskope, a cloud security platform that utilizes secure access service edge (SASE); HENNGE ONE, a SaaS authentication platform that provides secure access to cloud services and single sign-on functionality; HP Sure Click Enterprise, which provides endpoint protection with internet and web isolation apps; and SecureCube Access Check, a gateway-type privileged ID management solution. In addition, the company offers Imperva App Protect, a cloud based WAF and DDoS protection and operation service; Internal Risk Intelligence, an internal threat detection service; Privilege Management for Windows, an access management solution; RidgeBot, an AI-powered robot that offers implementation support and penetration testing service; GOOSEC, a SaaS-based web/online skimming prevention/detection tool; and SOCRadar, a security threat intelligence solution. Further, it provides IT consulting services for its GRC and security solutions, which include training services; implementation support for the design and construction of GRC-related tools; and system support services. The company was formerly known as NANAROQ Inc. and changed its name to GRCS Inc. in May 2018. GRCS Inc. was incorporated in 2005 and is headquartered in Chiyoda, Japan.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>グラッドキューブ</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>9561.T</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.glad-cube.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Software - Application</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>GLAD CUBE Inc. operates as an internet advertising agency in Japan. It operates through the Marketing DX Business and Technology Business segments. The company offers listing advertising management agency services, including listing advertisements, Facebook ads, Instagram ads, X (Twitter) ads, LINE ads, YouTube ads, application advertising, video advertisement production and operation, Apple search ads, DSP applications, Amazon ads, and beauty mail order/salon/clinic advertising operations, seminars, and free newsletter registration. It also provides production, analysis, and consulting services, such as website creation, vertical short drama production, access analysis, LPO/CRO consulting, LLMO/AIO countermeasures, and contract development services. In addition, the company offers SiTest, a tool for website analytics; SPAIA, an AI sports media platform; and SPAIA Horse Racing, a subscription-based service that extracts horse racing content. GLAD CUBE Inc. was incorporated in 2007 and is headquartered in Osaka, Japan.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>